<commit_message>
tedt data files mar 4 2024
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0011411VerifyUserWithTitleTAGOutsourcedContractor.xlsx
+++ b/TestData/LV_TMTT0011411VerifyUserWithTitleTAGOutsourcedContractor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31C5EEDC-9FC2-4DE2-A14A-537FDB799579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B10E0A-4282-4223-9BEF-DEF25C4DD196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="8" r:id="rId1"/>
@@ -933,7 +933,7 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>